<commit_message>
Tukar 3 soalan Imbuhan Apitan (Penilaian/Berlarian/Sebaiknya -> Pendidikan/Bersamaan/Secantiknya)
Ganti 3 soalan contoh dalam templat-imbuhan-apitan-7-soalan.xlsx atas
permintaan guru - "Pendidikan" (pe(n)-...-an, dasar "didik") sengaja
sertakan pilihan salah "Pe-" (tanpa nasal n) sbg distraktor yg relevan
secara pedagogi. Baki 4 soalan (Kehidupan, Kebersihan, Pertanian,
Mempercepatkan) kekal sama.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019P3uV9VgFDkRtAATVrH1g4
</commit_message>
<xml_diff>
--- a/public/templates/templat-imbuhan-apitan-7-soalan.xlsx
+++ b/public/templates/templat-imbuhan-apitan-7-soalan.xlsx
@@ -645,75 +645,75 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Penilaian</v>
+        <v>Pendidikan</v>
       </c>
       <c r="B5" t="str">
-        <v>nilai</v>
+        <v>didik</v>
       </c>
       <c r="C5" t="str">
-        <v>نيلاي</v>
+        <v>ديديك</v>
       </c>
       <c r="D5" t="str">
-        <v>Ber-</v>
+        <v>Pe-</v>
       </c>
       <c r="E5" t="str">
-        <v>بر</v>
+        <v>ڤ</v>
       </c>
       <c r="F5" t="str">
-        <v>Pe-</v>
+        <v>Pen-</v>
       </c>
       <c r="G5" t="str">
-        <v>ڤ</v>
+        <v>ڤن</v>
       </c>
       <c r="H5" t="str">
-        <v>Se-</v>
+        <v>Ke-</v>
       </c>
       <c r="I5" t="str">
-        <v>س</v>
+        <v>ک</v>
       </c>
       <c r="J5" t="str">
         <v>B</v>
       </c>
       <c r="K5" t="str">
+        <v>-kan</v>
+      </c>
+      <c r="L5" t="str">
+        <v>كن</v>
+      </c>
+      <c r="M5" t="str">
         <v>-an</v>
       </c>
-      <c r="L5" t="str">
+      <c r="N5" t="str">
         <v>ن</v>
       </c>
-      <c r="M5" t="str">
-        <v>-nya</v>
-      </c>
-      <c r="N5" t="str">
-        <v>ڽا</v>
-      </c>
       <c r="O5" t="str">
-        <v>-kan</v>
+        <v>-i</v>
       </c>
       <c r="P5" t="str">
-        <v>كن</v>
+        <v>ي</v>
       </c>
       <c r="Q5" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="R5" t="str">
-        <v>ڤنيلاين</v>
+        <v>ڤنديديكن</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Berlarian</v>
+        <v>Bersamaan</v>
       </c>
       <c r="B6" t="str">
-        <v>lari</v>
+        <v>sama</v>
       </c>
       <c r="C6" t="str">
-        <v>لاري</v>
+        <v>ساما</v>
       </c>
       <c r="D6" t="str">
-        <v>Pe-</v>
+        <v>Se-</v>
       </c>
       <c r="E6" t="str">
-        <v>ڤ</v>
+        <v>س</v>
       </c>
       <c r="F6" t="str">
         <v>Ber-</v>
@@ -731,16 +731,16 @@
         <v>B</v>
       </c>
       <c r="K6" t="str">
+        <v>-i</v>
+      </c>
+      <c r="L6" t="str">
+        <v>ي</v>
+      </c>
+      <c r="M6" t="str">
         <v>-kan</v>
       </c>
-      <c r="L6" t="str">
+      <c r="N6" t="str">
         <v>كن</v>
-      </c>
-      <c r="M6" t="str">
-        <v>-i</v>
-      </c>
-      <c r="N6" t="str">
-        <v>ي</v>
       </c>
       <c r="O6" t="str">
         <v>-an</v>
@@ -752,18 +752,18 @@
         <v>C</v>
       </c>
       <c r="R6" t="str">
-        <v>برلارين</v>
+        <v>برسامان</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Sebaiknya</v>
+        <v>Secantiknya</v>
       </c>
       <c r="B7" t="str">
-        <v>baik</v>
+        <v>cantik</v>
       </c>
       <c r="C7" t="str">
-        <v>بايك</v>
+        <v>چانتيك</v>
       </c>
       <c r="D7" t="str">
         <v>Se-</v>
@@ -772,10 +772,10 @@
         <v>س</v>
       </c>
       <c r="F7" t="str">
-        <v>Ke-</v>
+        <v>Pen-</v>
       </c>
       <c r="G7" t="str">
-        <v>ک</v>
+        <v>ڤن</v>
       </c>
       <c r="H7" t="str">
         <v>Ber-</v>
@@ -787,10 +787,10 @@
         <v>A</v>
       </c>
       <c r="K7" t="str">
-        <v>-an</v>
+        <v>-kan</v>
       </c>
       <c r="L7" t="str">
-        <v>ن</v>
+        <v>كن</v>
       </c>
       <c r="M7" t="str">
         <v>-nya</v>
@@ -799,16 +799,16 @@
         <v>ڽا</v>
       </c>
       <c r="O7" t="str">
-        <v>-kan</v>
+        <v>-an</v>
       </c>
       <c r="P7" t="str">
-        <v>كن</v>
+        <v>ن</v>
       </c>
       <c r="Q7" t="str">
         <v>B</v>
       </c>
       <c r="R7" t="str">
-        <v>سبايكڽا</v>
+        <v>سچانتيكڽا</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Tukar 2 soalan Imbuhan Apitan (Bersamaan/Secantiknya -> Pencerahan/Persembahan)
Ganti 2 soalan contoh dalam templat-imbuhan-apitan-7-soalan.xlsx atas
permintaan guru. Baki 5 soalan (Kehidupan, Kebersihan, Pertanian,
Pendidikan, Mempercepatkan) kekal sama.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019P3uV9VgFDkRtAATVrH1g4
</commit_message>
<xml_diff>
--- a/public/templates/templat-imbuhan-apitan-7-soalan.xlsx
+++ b/public/templates/templat-imbuhan-apitan-7-soalan.xlsx
@@ -701,25 +701,25 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Bersamaan</v>
+        <v>Pencerahan</v>
       </c>
       <c r="B6" t="str">
-        <v>sama</v>
+        <v>cerah</v>
       </c>
       <c r="C6" t="str">
-        <v>ساما</v>
+        <v>چراه</v>
       </c>
       <c r="D6" t="str">
-        <v>Se-</v>
+        <v>Pe-</v>
       </c>
       <c r="E6" t="str">
-        <v>س</v>
+        <v>ڤ</v>
       </c>
       <c r="F6" t="str">
-        <v>Ber-</v>
+        <v>Pen-</v>
       </c>
       <c r="G6" t="str">
-        <v>بر</v>
+        <v>ڤن</v>
       </c>
       <c r="H6" t="str">
         <v>Ke-</v>
@@ -731,16 +731,16 @@
         <v>B</v>
       </c>
       <c r="K6" t="str">
+        <v>-kan</v>
+      </c>
+      <c r="L6" t="str">
+        <v>كن</v>
+      </c>
+      <c r="M6" t="str">
         <v>-i</v>
       </c>
-      <c r="L6" t="str">
+      <c r="N6" t="str">
         <v>ي</v>
-      </c>
-      <c r="M6" t="str">
-        <v>-kan</v>
-      </c>
-      <c r="N6" t="str">
-        <v>كن</v>
       </c>
       <c r="O6" t="str">
         <v>-an</v>
@@ -752,51 +752,51 @@
         <v>C</v>
       </c>
       <c r="R6" t="str">
-        <v>برسامان</v>
+        <v>ڤنچراهن</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Secantiknya</v>
+        <v>Persembahan</v>
       </c>
       <c r="B7" t="str">
-        <v>cantik</v>
+        <v>sembah</v>
       </c>
       <c r="C7" t="str">
-        <v>چانتيك</v>
+        <v>سمباه</v>
       </c>
       <c r="D7" t="str">
-        <v>Se-</v>
+        <v>Ber-</v>
       </c>
       <c r="E7" t="str">
-        <v>س</v>
+        <v>بر</v>
       </c>
       <c r="F7" t="str">
-        <v>Pen-</v>
+        <v>Per-</v>
       </c>
       <c r="G7" t="str">
-        <v>ڤن</v>
+        <v>ڤر</v>
       </c>
       <c r="H7" t="str">
-        <v>Ber-</v>
+        <v>Memper-</v>
       </c>
       <c r="I7" t="str">
-        <v>بر</v>
+        <v>ممڤر</v>
       </c>
       <c r="J7" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="K7" t="str">
+        <v>-i</v>
+      </c>
+      <c r="L7" t="str">
+        <v>ي</v>
+      </c>
+      <c r="M7" t="str">
         <v>-kan</v>
       </c>
-      <c r="L7" t="str">
+      <c r="N7" t="str">
         <v>كن</v>
-      </c>
-      <c r="M7" t="str">
-        <v>-nya</v>
-      </c>
-      <c r="N7" t="str">
-        <v>ڽا</v>
       </c>
       <c r="O7" t="str">
         <v>-an</v>
@@ -805,10 +805,10 @@
         <v>ن</v>
       </c>
       <c r="Q7" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="R7" t="str">
-        <v>سچانتيكڽا</v>
+        <v>ڤرسمباهن</v>
       </c>
     </row>
     <row r="8">

</xml_diff>